<commit_message>
Addressed boundary solution issues
</commit_message>
<xml_diff>
--- a/input/employment_targets.xlsx
+++ b/input/employment_targets.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="14" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="28" uniqueCount="2">
   <si>
     <t>year</t>
   </si>
@@ -84,7 +84,7 @@
         <v>2011</v>
       </c>
       <c r="B2">
-        <v>0.86103755968005002</v>
+        <v>0.86039549023645712</v>
       </c>
     </row>
     <row r="3">
@@ -92,7 +92,7 @@
         <v>2012</v>
       </c>
       <c r="B3">
-        <v>0.86565293619847028</v>
+        <v>0.86553684320195845</v>
       </c>
     </row>
     <row r="4">
@@ -100,7 +100,7 @@
         <v>2013</v>
       </c>
       <c r="B4">
-        <v>0.87334042992501837</v>
+        <v>0.87333886016613127</v>
       </c>
     </row>
     <row r="5">
@@ -108,7 +108,7 @@
         <v>2014</v>
       </c>
       <c r="B5">
-        <v>0.89005194345721494</v>
+        <v>0.88980337145330857</v>
       </c>
     </row>
     <row r="6">
@@ -116,7 +116,7 @@
         <v>2015</v>
       </c>
       <c r="B6">
-        <v>0.89993866578562576</v>
+        <v>0.89903122500391819</v>
       </c>
     </row>
     <row r="7">
@@ -124,7 +124,7 @@
         <v>2016</v>
       </c>
       <c r="B7">
-        <v>0.90292797143888237</v>
+        <v>0.90199615953779644</v>
       </c>
     </row>
     <row r="8">
@@ -132,7 +132,7 @@
         <v>2017</v>
       </c>
       <c r="B8">
-        <v>0.90721826394684157</v>
+        <v>0.90557226178612993</v>
       </c>
     </row>
     <row r="9">
@@ -140,7 +140,7 @@
         <v>2018</v>
       </c>
       <c r="B9">
-        <v>0.91201898802956194</v>
+        <v>0.91044947834854817</v>
       </c>
     </row>
     <row r="10">
@@ -148,7 +148,7 @@
         <v>2019</v>
       </c>
       <c r="B10">
-        <v>0.91848291266177073</v>
+        <v>0.91760238972299813</v>
       </c>
     </row>
     <row r="11">
@@ -156,7 +156,7 @@
         <v>2020</v>
       </c>
       <c r="B11">
-        <v>0.91900914568017966</v>
+        <v>0.91542187874393632</v>
       </c>
     </row>
     <row r="12">
@@ -164,7 +164,7 @@
         <v>2021</v>
       </c>
       <c r="B12">
-        <v>0.92114164149452071</v>
+        <v>0.91797376338825565</v>
       </c>
     </row>
     <row r="13">
@@ -172,7 +172,7 @@
         <v>2022</v>
       </c>
       <c r="B13">
-        <v>0.93486006866447813</v>
+        <v>0.91772959177740587</v>
       </c>
     </row>
     <row r="14">
@@ -180,7 +180,7 @@
         <v>2023</v>
       </c>
       <c r="B14">
-        <v>0.93265139235348327</v>
+        <v>0.89808711590155499</v>
       </c>
     </row>
   </sheetData>
@@ -205,7 +205,7 @@
         <v>2011</v>
       </c>
       <c r="B2">
-        <v>0.50916259908360417</v>
+        <v>0.51220370836752216</v>
       </c>
     </row>
     <row r="3">
@@ -213,7 +213,7 @@
         <v>2012</v>
       </c>
       <c r="B3">
-        <v>0.50930277081592867</v>
+        <v>0.50609286734887104</v>
       </c>
     </row>
     <row r="4">
@@ -221,7 +221,7 @@
         <v>2013</v>
       </c>
       <c r="B4">
-        <v>0.52308518171117491</v>
+        <v>0.52162516980654317</v>
       </c>
     </row>
     <row r="5">
@@ -229,7 +229,7 @@
         <v>2014</v>
       </c>
       <c r="B5">
-        <v>0.54901652519255928</v>
+        <v>0.5472354417236307</v>
       </c>
     </row>
     <row r="6">
@@ -237,7 +237,7 @@
         <v>2015</v>
       </c>
       <c r="B6">
-        <v>0.54361644921178498</v>
+        <v>0.54262361056790287</v>
       </c>
     </row>
     <row r="7">
@@ -245,7 +245,7 @@
         <v>2016</v>
       </c>
       <c r="B7">
-        <v>0.54944855403904691</v>
+        <v>0.54944960497911599</v>
       </c>
     </row>
     <row r="8">
@@ -253,7 +253,7 @@
         <v>2017</v>
       </c>
       <c r="B8">
-        <v>0.53930619518798029</v>
+        <v>0.53837190826757053</v>
       </c>
     </row>
     <row r="9">
@@ -261,7 +261,7 @@
         <v>2018</v>
       </c>
       <c r="B9">
-        <v>0.54464825905109293</v>
+        <v>0.53730892446494438</v>
       </c>
     </row>
     <row r="10">
@@ -269,7 +269,7 @@
         <v>2019</v>
       </c>
       <c r="B10">
-        <v>0.54590154269031532</v>
+        <v>0.54022372042418654</v>
       </c>
     </row>
     <row r="11">
@@ -277,7 +277,7 @@
         <v>2020</v>
       </c>
       <c r="B11">
-        <v>0.5526845420360188</v>
+        <v>0.54988897544427096</v>
       </c>
     </row>
     <row r="12">
@@ -285,7 +285,7 @@
         <v>2021</v>
       </c>
       <c r="B12">
-        <v>0.54236302578780049</v>
+        <v>0.53821147608486786</v>
       </c>
     </row>
     <row r="13">
@@ -293,7 +293,7 @@
         <v>2022</v>
       </c>
       <c r="B13">
-        <v>0.54267555033690795</v>
+        <v>0.53822494202667048</v>
       </c>
     </row>
     <row r="14">
@@ -301,7 +301,7 @@
         <v>2023</v>
       </c>
       <c r="B14">
-        <v>0.54934185941202596</v>
+        <v>0.57308246103213423</v>
       </c>
     </row>
   </sheetData>
@@ -326,7 +326,7 @@
         <v>2011</v>
       </c>
       <c r="B2">
-        <v>0.52424514222099061</v>
+        <v>0.5256034710997578</v>
       </c>
     </row>
     <row r="3">
@@ -334,7 +334,7 @@
         <v>2012</v>
       </c>
       <c r="B3">
-        <v>0.5297646568214166</v>
+        <v>0.53190535335554368</v>
       </c>
     </row>
     <row r="4">
@@ -342,7 +342,7 @@
         <v>2013</v>
       </c>
       <c r="B4">
-        <v>0.55220348919174123</v>
+        <v>0.5561772080232934</v>
       </c>
     </row>
     <row r="5">
@@ -350,7 +350,7 @@
         <v>2014</v>
       </c>
       <c r="B5">
-        <v>0.56445361032167196</v>
+        <v>0.56475736609552796</v>
       </c>
     </row>
     <row r="6">
@@ -358,7 +358,7 @@
         <v>2015</v>
       </c>
       <c r="B6">
-        <v>0.57754838790736829</v>
+        <v>0.57478238567069184</v>
       </c>
     </row>
     <row r="7">
@@ -366,7 +366,7 @@
         <v>2016</v>
       </c>
       <c r="B7">
-        <v>0.57988539212111645</v>
+        <v>0.58052633470130843</v>
       </c>
     </row>
     <row r="8">
@@ -374,7 +374,7 @@
         <v>2017</v>
       </c>
       <c r="B8">
-        <v>0.5525876078384665</v>
+        <v>0.55390611514386168</v>
       </c>
     </row>
     <row r="9">
@@ -382,7 +382,7 @@
         <v>2018</v>
       </c>
       <c r="B9">
-        <v>0.54796118140361605</v>
+        <v>0.54592493660333552</v>
       </c>
     </row>
     <row r="10">
@@ -390,7 +390,7 @@
         <v>2019</v>
       </c>
       <c r="B10">
-        <v>0.54173937355852486</v>
+        <v>0.53163699870605541</v>
       </c>
     </row>
     <row r="11">
@@ -398,7 +398,7 @@
         <v>2020</v>
       </c>
       <c r="B11">
-        <v>0.5206936686584952</v>
+        <v>0.51102844420261284</v>
       </c>
     </row>
     <row r="12">
@@ -406,7 +406,7 @@
         <v>2021</v>
       </c>
       <c r="B12">
-        <v>0.51572152506838742</v>
+        <v>0.51264287652516671</v>
       </c>
     </row>
     <row r="13">
@@ -414,7 +414,7 @@
         <v>2022</v>
       </c>
       <c r="B13">
-        <v>0.59843645588015859</v>
+        <v>0.54231629380257707</v>
       </c>
     </row>
     <row r="14">
@@ -422,7 +422,7 @@
         <v>2023</v>
       </c>
       <c r="B14">
-        <v>0.54299119391420037</v>
+        <v>0.54685537387931238</v>
       </c>
     </row>
   </sheetData>
@@ -447,7 +447,7 @@
         <v>2011</v>
       </c>
       <c r="B2">
-        <v>0.39556045345564655</v>
+        <v>0.70332673058801953</v>
       </c>
     </row>
     <row r="3">
@@ -455,7 +455,7 @@
         <v>2012</v>
       </c>
       <c r="B3">
-        <v>0.39826887032633312</v>
+        <v>0.71362107370227112</v>
       </c>
     </row>
     <row r="4">
@@ -463,7 +463,7 @@
         <v>2013</v>
       </c>
       <c r="B4">
-        <v>0.41788999233132329</v>
+        <v>0.74324722315718617</v>
       </c>
     </row>
     <row r="5">
@@ -471,7 +471,7 @@
         <v>2014</v>
       </c>
       <c r="B5">
-        <v>0.41641254321738624</v>
+        <v>0.75330174270165895</v>
       </c>
     </row>
     <row r="6">
@@ -479,7 +479,7 @@
         <v>2015</v>
       </c>
       <c r="B6">
-        <v>0.43288978646377752</v>
+        <v>0.74543035750704934</v>
       </c>
     </row>
     <row r="7">
@@ -487,7 +487,7 @@
         <v>2016</v>
       </c>
       <c r="B7">
-        <v>0.45189418379574153</v>
+        <v>0.80622828282828285</v>
       </c>
     </row>
     <row r="8">
@@ -495,7 +495,7 @@
         <v>2017</v>
       </c>
       <c r="B8">
-        <v>0.45364344178605082</v>
+        <v>0.80111241131800182</v>
       </c>
     </row>
     <row r="9">
@@ -503,7 +503,7 @@
         <v>2018</v>
       </c>
       <c r="B9">
-        <v>0.45865757513278943</v>
+        <v>0.81986761541930764</v>
       </c>
     </row>
     <row r="10">
@@ -511,7 +511,7 @@
         <v>2019</v>
       </c>
       <c r="B10">
-        <v>0.47317042277347493</v>
+        <v>0.83828124367780332</v>
       </c>
     </row>
     <row r="11">
@@ -519,7 +519,7 @@
         <v>2020</v>
       </c>
       <c r="B11">
-        <v>0.46809655995986466</v>
+        <v>0.8539477290141444</v>
       </c>
     </row>
     <row r="12">
@@ -527,7 +527,7 @@
         <v>2021</v>
       </c>
       <c r="B12">
-        <v>0.46820351031329249</v>
+        <v>0.84489922396840822</v>
       </c>
     </row>
     <row r="13">
@@ -535,7 +535,7 @@
         <v>2022</v>
       </c>
       <c r="B13">
-        <v>0.46942323493860777</v>
+        <v>0.87577709165987916</v>
       </c>
     </row>
     <row r="14">
@@ -543,7 +543,7 @@
         <v>2023</v>
       </c>
       <c r="B14">
-        <v>0.45820714330329332</v>
+        <v>0.78522593714692146</v>
       </c>
     </row>
   </sheetData>
@@ -568,7 +568,7 @@
         <v>2011</v>
       </c>
       <c r="B2">
-        <v>0.50906604919978893</v>
+        <v>0.88109057219593834</v>
       </c>
     </row>
     <row r="3">
@@ -576,7 +576,7 @@
         <v>2012</v>
       </c>
       <c r="B3">
-        <v>0.50437075567114575</v>
+        <v>0.8690482364373544</v>
       </c>
     </row>
     <row r="4">
@@ -584,7 +584,7 @@
         <v>2013</v>
       </c>
       <c r="B4">
-        <v>0.50772668179019009</v>
+        <v>0.88090220029991562</v>
       </c>
     </row>
     <row r="5">
@@ -592,7 +592,7 @@
         <v>2014</v>
       </c>
       <c r="B5">
-        <v>0.51786184005593128</v>
+        <v>0.87079652990766343</v>
       </c>
     </row>
     <row r="6">
@@ -600,7 +600,7 @@
         <v>2015</v>
       </c>
       <c r="B6">
-        <v>0.54892632878551184</v>
+        <v>0.89160821111255328</v>
       </c>
     </row>
     <row r="7">
@@ -608,7 +608,7 @@
         <v>2016</v>
       </c>
       <c r="B7">
-        <v>0.56344976547872083</v>
+        <v>0.91560860881279604</v>
       </c>
     </row>
     <row r="8">
@@ -616,7 +616,7 @@
         <v>2017</v>
       </c>
       <c r="B8">
-        <v>0.54977685502827922</v>
+        <v>0.90649600258283003</v>
       </c>
     </row>
     <row r="9">
@@ -624,7 +624,7 @@
         <v>2018</v>
       </c>
       <c r="B9">
-        <v>0.53292474255669975</v>
+        <v>0.90339643407616077</v>
       </c>
     </row>
     <row r="10">
@@ -632,7 +632,7 @@
         <v>2019</v>
       </c>
       <c r="B10">
-        <v>0.58288034104237252</v>
+        <v>0.93468859322920972</v>
       </c>
     </row>
     <row r="11">
@@ -640,7 +640,7 @@
         <v>2020</v>
       </c>
       <c r="B11">
-        <v>0.57159502490313252</v>
+        <v>0.93070206055223348</v>
       </c>
     </row>
     <row r="12">
@@ -648,7 +648,7 @@
         <v>2021</v>
       </c>
       <c r="B12">
-        <v>0.56248281380715093</v>
+        <v>0.94149841798207434</v>
       </c>
     </row>
     <row r="13">
@@ -656,7 +656,7 @@
         <v>2022</v>
       </c>
       <c r="B13">
-        <v>0.55988118695081046</v>
+        <v>0.91827223331881125</v>
       </c>
     </row>
     <row r="14">
@@ -664,7 +664,7 @@
         <v>2023</v>
       </c>
       <c r="B14">
-        <v>0.576489694027432</v>
+        <v>0.93221374920615219</v>
       </c>
     </row>
   </sheetData>
@@ -689,7 +689,7 @@
         <v>2011</v>
       </c>
       <c r="B2">
-        <v>0.42493296556276605</v>
+        <v>0.42127482893775326</v>
       </c>
     </row>
     <row r="3">
@@ -697,7 +697,7 @@
         <v>2012</v>
       </c>
       <c r="B3">
-        <v>0.41552900265172893</v>
+        <v>0.41140425015620114</v>
       </c>
     </row>
     <row r="4">
@@ -705,7 +705,7 @@
         <v>2013</v>
       </c>
       <c r="B4">
-        <v>0.43637149307617717</v>
+        <v>0.42995845340983302</v>
       </c>
     </row>
     <row r="5">
@@ -713,7 +713,7 @@
         <v>2014</v>
       </c>
       <c r="B5">
-        <v>0.4392160207423581</v>
+        <v>0.43282612682370203</v>
       </c>
     </row>
     <row r="6">
@@ -721,7 +721,7 @@
         <v>2015</v>
       </c>
       <c r="B6">
-        <v>0.45017675231064397</v>
+        <v>0.44208310617813035</v>
       </c>
     </row>
     <row r="7">
@@ -729,7 +729,7 @@
         <v>2016</v>
       </c>
       <c r="B7">
-        <v>0.45498139340201532</v>
+        <v>0.44517711913597557</v>
       </c>
     </row>
     <row r="8">
@@ -737,7 +737,7 @@
         <v>2017</v>
       </c>
       <c r="B8">
-        <v>0.46380899913592816</v>
+        <v>0.45419570757468758</v>
       </c>
     </row>
     <row r="9">
@@ -745,7 +745,7 @@
         <v>2018</v>
       </c>
       <c r="B9">
-        <v>0.46073257871240159</v>
+        <v>0.45065641725778849</v>
       </c>
     </row>
     <row r="10">
@@ -753,7 +753,7 @@
         <v>2019</v>
       </c>
       <c r="B10">
-        <v>0.45519037857316585</v>
+        <v>0.44371813085715239</v>
       </c>
     </row>
     <row r="11">
@@ -761,7 +761,7 @@
         <v>2020</v>
       </c>
       <c r="B11">
-        <v>0.45645113009870603</v>
+        <v>0.44281548466086768</v>
       </c>
     </row>
     <row r="12">
@@ -769,7 +769,7 @@
         <v>2021</v>
       </c>
       <c r="B12">
-        <v>0.45898196380860801</v>
+        <v>0.44498860993488526</v>
       </c>
     </row>
     <row r="13">
@@ -777,7 +777,7 @@
         <v>2022</v>
       </c>
       <c r="B13">
-        <v>0.46799998752682881</v>
+        <v>0.45292141535099589</v>
       </c>
     </row>
     <row r="14">
@@ -785,7 +785,7 @@
         <v>2023</v>
       </c>
       <c r="B14">
-        <v>0.47588068836384528</v>
+        <v>0.47013399643946252</v>
       </c>
     </row>
   </sheetData>
@@ -810,7 +810,7 @@
         <v>2011</v>
       </c>
       <c r="B2">
-        <v>0.48237464081683645</v>
+        <v>0.47583382100076582</v>
       </c>
     </row>
     <row r="3">
@@ -818,7 +818,7 @@
         <v>2012</v>
       </c>
       <c r="B3">
-        <v>0.47103636423616307</v>
+        <v>0.46141730655853214</v>
       </c>
     </row>
     <row r="4">
@@ -826,7 +826,7 @@
         <v>2013</v>
       </c>
       <c r="B4">
-        <v>0.48403135220541249</v>
+        <v>0.47274739467355481</v>
       </c>
     </row>
     <row r="5">
@@ -834,7 +834,7 @@
         <v>2014</v>
       </c>
       <c r="B5">
-        <v>0.49370142498373548</v>
+        <v>0.47963372180757602</v>
       </c>
     </row>
     <row r="6">
@@ -842,7 +842,7 @@
         <v>2015</v>
       </c>
       <c r="B6">
-        <v>0.49022220287710289</v>
+        <v>0.47728646381028406</v>
       </c>
     </row>
     <row r="7">
@@ -850,7 +850,7 @@
         <v>2016</v>
       </c>
       <c r="B7">
-        <v>0.4958887579640005</v>
+        <v>0.48187730838587955</v>
       </c>
     </row>
     <row r="8">
@@ -858,7 +858,7 @@
         <v>2017</v>
       </c>
       <c r="B8">
-        <v>0.48631680371954544</v>
+        <v>0.4721974661313435</v>
       </c>
     </row>
     <row r="9">
@@ -866,7 +866,7 @@
         <v>2018</v>
       </c>
       <c r="B9">
-        <v>0.47856452699154889</v>
+        <v>0.46186711889490872</v>
       </c>
     </row>
     <row r="10">
@@ -874,7 +874,7 @@
         <v>2019</v>
       </c>
       <c r="B10">
-        <v>0.48611504211950518</v>
+        <v>0.47054426414387607</v>
       </c>
     </row>
     <row r="11">
@@ -882,7 +882,7 @@
         <v>2020</v>
       </c>
       <c r="B11">
-        <v>0.48476239547710198</v>
+        <v>0.46481409041604849</v>
       </c>
     </row>
     <row r="12">
@@ -890,7 +890,7 @@
         <v>2021</v>
       </c>
       <c r="B12">
-        <v>0.49728963079573468</v>
+        <v>0.47764394229936535</v>
       </c>
     </row>
     <row r="13">
@@ -898,7 +898,7 @@
         <v>2022</v>
       </c>
       <c r="B13">
-        <v>0.49660798739828316</v>
+        <v>0.50992956293613689</v>
       </c>
     </row>
     <row r="14">
@@ -906,7 +906,7 @@
         <v>2023</v>
       </c>
       <c r="B14">
-        <v>0.48352007275312292</v>
+        <v>0.52898311289960343</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added care need flag to do-file.
</commit_message>
<xml_diff>
--- a/input/employment_targets.xlsx
+++ b/input/employment_targets.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="28" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="140" uniqueCount="2">
   <si>
     <t>year</t>
   </si>
@@ -116,7 +116,7 @@
         <v>2015</v>
       </c>
       <c r="B6">
-        <v>0.89903122500391819</v>
+        <v>0.899079853821525</v>
       </c>
     </row>
     <row r="7">
@@ -124,7 +124,7 @@
         <v>2016</v>
       </c>
       <c r="B7">
-        <v>0.90199615953779644</v>
+        <v>0.90206057810487217</v>
       </c>
     </row>
     <row r="8">
@@ -132,7 +132,7 @@
         <v>2017</v>
       </c>
       <c r="B8">
-        <v>0.90557226178612993</v>
+        <v>0.90549711853962811</v>
       </c>
     </row>
     <row r="9">
@@ -140,7 +140,7 @@
         <v>2018</v>
       </c>
       <c r="B9">
-        <v>0.91044947834854817</v>
+        <v>0.91066305658584679</v>
       </c>
     </row>
     <row r="10">
@@ -148,7 +148,7 @@
         <v>2019</v>
       </c>
       <c r="B10">
-        <v>0.91760238972299813</v>
+        <v>0.91759601842003469</v>
       </c>
     </row>
     <row r="11">
@@ -156,7 +156,7 @@
         <v>2020</v>
       </c>
       <c r="B11">
-        <v>0.91542187874393632</v>
+        <v>0.91548053277542307</v>
       </c>
     </row>
     <row r="12">
@@ -164,7 +164,7 @@
         <v>2021</v>
       </c>
       <c r="B12">
-        <v>0.91797376338825565</v>
+        <v>0.91786256873220062</v>
       </c>
     </row>
     <row r="13">
@@ -172,7 +172,7 @@
         <v>2022</v>
       </c>
       <c r="B13">
-        <v>0.91772959177740587</v>
+        <v>0.91757613060603349</v>
       </c>
     </row>
     <row r="14">
@@ -479,7 +479,7 @@
         <v>2015</v>
       </c>
       <c r="B6">
-        <v>0.74543035750704934</v>
+        <v>0.74349169078193489</v>
       </c>
     </row>
     <row r="7">
@@ -487,7 +487,7 @@
         <v>2016</v>
       </c>
       <c r="B7">
-        <v>0.80622828282828285</v>
+        <v>0.80226067113929578</v>
       </c>
     </row>
     <row r="8">
@@ -495,7 +495,7 @@
         <v>2017</v>
       </c>
       <c r="B8">
-        <v>0.80111241131800182</v>
+        <v>0.80026172215143476</v>
       </c>
     </row>
     <row r="9">
@@ -503,7 +503,7 @@
         <v>2018</v>
       </c>
       <c r="B9">
-        <v>0.81986761541930764</v>
+        <v>0.81810829974119437</v>
       </c>
     </row>
     <row r="10">
@@ -511,7 +511,7 @@
         <v>2019</v>
       </c>
       <c r="B10">
-        <v>0.83828124367780332</v>
+        <v>0.83669398111411242</v>
       </c>
     </row>
     <row r="11">
@@ -519,7 +519,7 @@
         <v>2020</v>
       </c>
       <c r="B11">
-        <v>0.8539477290141444</v>
+        <v>0.85238231281962984</v>
       </c>
     </row>
     <row r="12">
@@ -527,7 +527,7 @@
         <v>2021</v>
       </c>
       <c r="B12">
-        <v>0.84489922396840822</v>
+        <v>0.84502580094992652</v>
       </c>
     </row>
     <row r="13">
@@ -535,7 +535,7 @@
         <v>2022</v>
       </c>
       <c r="B13">
-        <v>0.87577709165987916</v>
+        <v>0.87859406500018256</v>
       </c>
     </row>
     <row r="14">
@@ -600,7 +600,7 @@
         <v>2015</v>
       </c>
       <c r="B6">
-        <v>0.89160821111255328</v>
+        <v>0.89040469754869978</v>
       </c>
     </row>
     <row r="7">
@@ -608,7 +608,7 @@
         <v>2016</v>
       </c>
       <c r="B7">
-        <v>0.91560860881279604</v>
+        <v>0.91386524975670314</v>
       </c>
     </row>
     <row r="8">
@@ -616,7 +616,7 @@
         <v>2017</v>
       </c>
       <c r="B8">
-        <v>0.90649600258283003</v>
+        <v>0.9052754229528639</v>
       </c>
     </row>
     <row r="9">
@@ -624,7 +624,7 @@
         <v>2018</v>
       </c>
       <c r="B9">
-        <v>0.90339643407616077</v>
+        <v>0.90395412484499194</v>
       </c>
     </row>
     <row r="10">
@@ -632,7 +632,7 @@
         <v>2019</v>
       </c>
       <c r="B10">
-        <v>0.93468859322920972</v>
+        <v>0.93333109757233623</v>
       </c>
     </row>
     <row r="11">
@@ -640,7 +640,7 @@
         <v>2020</v>
       </c>
       <c r="B11">
-        <v>0.93070206055223348</v>
+        <v>0.92899330803420543</v>
       </c>
     </row>
     <row r="12">
@@ -648,7 +648,7 @@
         <v>2021</v>
       </c>
       <c r="B12">
-        <v>0.94149841798207434</v>
+        <v>0.94142725087816603</v>
       </c>
     </row>
     <row r="13">
@@ -656,7 +656,7 @@
         <v>2022</v>
       </c>
       <c r="B13">
-        <v>0.91827223331881125</v>
+        <v>0.91857422607721817</v>
       </c>
     </row>
     <row r="14">

</xml_diff>

<commit_message>
Updated employment alignment targets file, employment_targets.xlsx
</commit_message>
<xml_diff>
--- a/input/employment_targets.xlsx
+++ b/input/employment_targets.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="196" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="210" uniqueCount="2">
   <si>
     <t>year</t>
   </si>
@@ -84,7 +84,7 @@
         <v>2011</v>
       </c>
       <c r="B2">
-        <v>0.82196283228976819</v>
+        <v>0.82194953105605106</v>
       </c>
     </row>
     <row r="3">
@@ -92,7 +92,7 @@
         <v>2012</v>
       </c>
       <c r="B3">
-        <v>0.8263734620131602</v>
+        <v>0.82636904787711407</v>
       </c>
     </row>
     <row r="4">
@@ -100,7 +100,7 @@
         <v>2013</v>
       </c>
       <c r="B4">
-        <v>0.83503180512283726</v>
+        <v>0.83501949671114184</v>
       </c>
     </row>
     <row r="5">
@@ -108,7 +108,7 @@
         <v>2014</v>
       </c>
       <c r="B5">
-        <v>0.84872929309402723</v>
+        <v>0.84873588283804424</v>
       </c>
     </row>
     <row r="6">
@@ -116,7 +116,7 @@
         <v>2015</v>
       </c>
       <c r="B6">
-        <v>0.85477355018134593</v>
+        <v>0.85473546119865018</v>
       </c>
     </row>
     <row r="7">
@@ -124,7 +124,7 @@
         <v>2016</v>
       </c>
       <c r="B7">
-        <v>0.86022855882154659</v>
+        <v>0.8602126045694507</v>
       </c>
     </row>
     <row r="8">
@@ -132,7 +132,7 @@
         <v>2017</v>
       </c>
       <c r="B8">
-        <v>0.86116745205721168</v>
+        <v>0.86120776022503698</v>
       </c>
     </row>
     <row r="9">
@@ -140,7 +140,7 @@
         <v>2018</v>
       </c>
       <c r="B9">
-        <v>0.86785875236385246</v>
+        <v>0.86780763455897414</v>
       </c>
     </row>
     <row r="10">
@@ -148,7 +148,7 @@
         <v>2019</v>
       </c>
       <c r="B10">
-        <v>0.87374159615658542</v>
+        <v>0.87359700031119292</v>
       </c>
     </row>
     <row r="11">
@@ -156,7 +156,7 @@
         <v>2020</v>
       </c>
       <c r="B11">
-        <v>0.87556922627861711</v>
+        <v>0.87543897717978825</v>
       </c>
     </row>
     <row r="12">
@@ -164,7 +164,7 @@
         <v>2021</v>
       </c>
       <c r="B12">
-        <v>0.87758220527054198</v>
+        <v>0.87764181222899407</v>
       </c>
     </row>
     <row r="13">
@@ -172,7 +172,7 @@
         <v>2022</v>
       </c>
       <c r="B13">
-        <v>0.87117290567931704</v>
+        <v>0.87120186432025259</v>
       </c>
     </row>
     <row r="14">
@@ -180,7 +180,7 @@
         <v>2023</v>
       </c>
       <c r="B14">
-        <v>0.85418283993132527</v>
+        <v>0.85434281192935657</v>
       </c>
     </row>
   </sheetData>
@@ -205,7 +205,7 @@
         <v>2011</v>
       </c>
       <c r="B2">
-        <v>0.51238342740352727</v>
+        <v>0.51222149299376851</v>
       </c>
     </row>
     <row r="3">
@@ -213,7 +213,7 @@
         <v>2012</v>
       </c>
       <c r="B3">
-        <v>0.50608932818183383</v>
+        <v>0.50614819870505989</v>
       </c>
     </row>
     <row r="4">
@@ -221,7 +221,7 @@
         <v>2013</v>
       </c>
       <c r="B4">
-        <v>0.52174309687748743</v>
+        <v>0.52169514798729977</v>
       </c>
     </row>
     <row r="5">
@@ -229,7 +229,7 @@
         <v>2014</v>
       </c>
       <c r="B5">
-        <v>0.54707419047893657</v>
+        <v>0.54717760594146925</v>
       </c>
     </row>
     <row r="6">
@@ -237,7 +237,7 @@
         <v>2015</v>
       </c>
       <c r="B6">
-        <v>0.54261801305254231</v>
+        <v>0.5426061284255137</v>
       </c>
     </row>
     <row r="7">
@@ -245,7 +245,7 @@
         <v>2016</v>
       </c>
       <c r="B7">
-        <v>0.549444135041535</v>
+        <v>0.54929338426341023</v>
       </c>
     </row>
     <row r="8">
@@ -253,7 +253,7 @@
         <v>2017</v>
       </c>
       <c r="B8">
-        <v>0.53867440027030067</v>
+        <v>0.53846717211835637</v>
       </c>
     </row>
     <row r="9">
@@ -261,7 +261,7 @@
         <v>2018</v>
       </c>
       <c r="B9">
-        <v>0.53730890794618835</v>
+        <v>0.53760751533573414</v>
       </c>
     </row>
     <row r="10">
@@ -269,7 +269,7 @@
         <v>2019</v>
       </c>
       <c r="B10">
-        <v>0.54023621458905025</v>
+        <v>0.54032938088536064</v>
       </c>
     </row>
     <row r="11">
@@ -277,7 +277,7 @@
         <v>2020</v>
       </c>
       <c r="B11">
-        <v>0.54988459085533081</v>
+        <v>0.55019853924087125</v>
       </c>
     </row>
     <row r="12">
@@ -285,7 +285,7 @@
         <v>2021</v>
       </c>
       <c r="B12">
-        <v>0.53821639288769818</v>
+        <v>0.53827188015055483</v>
       </c>
     </row>
     <row r="13">
@@ -293,7 +293,7 @@
         <v>2022</v>
       </c>
       <c r="B13">
-        <v>0.53803079640521401</v>
+        <v>0.5382469728746202</v>
       </c>
     </row>
     <row r="14">
@@ -301,7 +301,7 @@
         <v>2023</v>
       </c>
       <c r="B14">
-        <v>0.57309638811663066</v>
+        <v>0.57322517483795643</v>
       </c>
     </row>
   </sheetData>
@@ -326,7 +326,7 @@
         <v>2011</v>
       </c>
       <c r="B2">
-        <v>0.5256081667589505</v>
+        <v>0.52560224211559758</v>
       </c>
     </row>
     <row r="3">
@@ -334,7 +334,7 @@
         <v>2012</v>
       </c>
       <c r="B3">
-        <v>0.53190573453478229</v>
+        <v>0.53197217608066516</v>
       </c>
     </row>
     <row r="4">
@@ -342,7 +342,7 @@
         <v>2013</v>
       </c>
       <c r="B4">
-        <v>0.5561863299780403</v>
+        <v>0.55614815923255179</v>
       </c>
     </row>
     <row r="5">
@@ -350,7 +350,7 @@
         <v>2014</v>
       </c>
       <c r="B5">
-        <v>0.56475260792437676</v>
+        <v>0.56470381636554112</v>
       </c>
     </row>
     <row r="6">
@@ -358,7 +358,7 @@
         <v>2015</v>
       </c>
       <c r="B6">
-        <v>0.57477798331485597</v>
+        <v>0.57476835128938031</v>
       </c>
     </row>
     <row r="7">
@@ -366,7 +366,7 @@
         <v>2016</v>
       </c>
       <c r="B7">
-        <v>0.58051865191440433</v>
+        <v>0.58061529176847637</v>
       </c>
     </row>
     <row r="8">
@@ -374,7 +374,7 @@
         <v>2017</v>
       </c>
       <c r="B8">
-        <v>0.5537474667771729</v>
+        <v>0.55370879994187261</v>
       </c>
     </row>
     <row r="9">
@@ -382,7 +382,7 @@
         <v>2018</v>
       </c>
       <c r="B9">
-        <v>0.54592269338929289</v>
+        <v>0.54541360532645933</v>
       </c>
     </row>
     <row r="10">
@@ -390,7 +390,7 @@
         <v>2019</v>
       </c>
       <c r="B10">
-        <v>0.53164663756530273</v>
+        <v>0.53117912591178562</v>
       </c>
     </row>
     <row r="11">
@@ -398,7 +398,7 @@
         <v>2020</v>
       </c>
       <c r="B11">
-        <v>0.51113709006815589</v>
+        <v>0.51095228369600443</v>
       </c>
     </row>
     <row r="12">
@@ -406,7 +406,7 @@
         <v>2021</v>
       </c>
       <c r="B12">
-        <v>0.51289330043723869</v>
+        <v>0.5130523068280014</v>
       </c>
     </row>
     <row r="13">
@@ -414,7 +414,7 @@
         <v>2022</v>
       </c>
       <c r="B13">
-        <v>0.54231482992222702</v>
+        <v>0.54232485796604457</v>
       </c>
     </row>
     <row r="14">
@@ -422,7 +422,7 @@
         <v>2023</v>
       </c>
       <c r="B14">
-        <v>0.54686656700889003</v>
+        <v>0.54728386631073978</v>
       </c>
     </row>
   </sheetData>
@@ -447,7 +447,7 @@
         <v>2011</v>
       </c>
       <c r="B2">
-        <v>0.37383525377704374</v>
+        <v>0.37384178456294531</v>
       </c>
     </row>
     <row r="3">
@@ -455,7 +455,7 @@
         <v>2012</v>
       </c>
       <c r="B3">
-        <v>0.38004918524548353</v>
+        <v>0.38005658699292066</v>
       </c>
     </row>
     <row r="4">
@@ -463,7 +463,7 @@
         <v>2013</v>
       </c>
       <c r="B4">
-        <v>0.38563002731646456</v>
+        <v>0.38564217656209487</v>
       </c>
     </row>
     <row r="5">
@@ -471,7 +471,7 @@
         <v>2014</v>
       </c>
       <c r="B5">
-        <v>0.38543593434287865</v>
+        <v>0.38543356372670229</v>
       </c>
     </row>
     <row r="6">
@@ -479,7 +479,7 @@
         <v>2015</v>
       </c>
       <c r="B6">
-        <v>0.38543924049685907</v>
+        <v>0.38545134862145075</v>
       </c>
     </row>
     <row r="7">
@@ -487,7 +487,7 @@
         <v>2016</v>
       </c>
       <c r="B7">
-        <v>0.40353282232065935</v>
+        <v>0.40354195390275061</v>
       </c>
     </row>
     <row r="8">
@@ -495,7 +495,7 @@
         <v>2017</v>
       </c>
       <c r="B8">
-        <v>0.39662403997863549</v>
+        <v>0.39662227110957793</v>
       </c>
     </row>
     <row r="9">
@@ -503,7 +503,7 @@
         <v>2018</v>
       </c>
       <c r="B9">
-        <v>0.38103707638688922</v>
+        <v>0.38106593589434762</v>
       </c>
     </row>
     <row r="10">
@@ -511,7 +511,7 @@
         <v>2019</v>
       </c>
       <c r="B10">
-        <v>0.39432077963579154</v>
+        <v>0.39433666380899263</v>
       </c>
     </row>
     <row r="11">
@@ -519,7 +519,7 @@
         <v>2020</v>
       </c>
       <c r="B11">
-        <v>0.39395894675582882</v>
+        <v>0.39419591944290849</v>
       </c>
     </row>
     <row r="12">
@@ -527,7 +527,7 @@
         <v>2021</v>
       </c>
       <c r="B12">
-        <v>0.39808109818429638</v>
+        <v>0.39809788164553633</v>
       </c>
     </row>
     <row r="13">
@@ -535,7 +535,7 @@
         <v>2022</v>
       </c>
       <c r="B13">
-        <v>0.41334265935329767</v>
+        <v>0.4133664269810563</v>
       </c>
     </row>
     <row r="14">
@@ -543,7 +543,7 @@
         <v>2023</v>
       </c>
       <c r="B14">
-        <v>0.38301264874520991</v>
+        <v>0.38314371198891167</v>
       </c>
     </row>
   </sheetData>
@@ -568,7 +568,7 @@
         <v>2011</v>
       </c>
       <c r="B2">
-        <v>0.42098114227740358</v>
+        <v>0.42099066545345665</v>
       </c>
     </row>
     <row r="3">
@@ -576,7 +576,7 @@
         <v>2012</v>
       </c>
       <c r="B3">
-        <v>0.43463852442062284</v>
+        <v>0.43454227778103005</v>
       </c>
     </row>
     <row r="4">
@@ -584,7 +584,7 @@
         <v>2013</v>
       </c>
       <c r="B4">
-        <v>0.44253497132011671</v>
+        <v>0.44253459907822163</v>
       </c>
     </row>
     <row r="5">
@@ -592,7 +592,7 @@
         <v>2014</v>
       </c>
       <c r="B5">
-        <v>0.44003282009205008</v>
+        <v>0.44003513062598865</v>
       </c>
     </row>
     <row r="6">
@@ -600,7 +600,7 @@
         <v>2015</v>
       </c>
       <c r="B6">
-        <v>0.44507840338898158</v>
+        <v>0.44508887219360893</v>
       </c>
     </row>
     <row r="7">
@@ -608,7 +608,7 @@
         <v>2016</v>
       </c>
       <c r="B7">
-        <v>0.45891012528402814</v>
+        <v>0.45890062520192948</v>
       </c>
     </row>
     <row r="8">
@@ -616,7 +616,7 @@
         <v>2017</v>
       </c>
       <c r="B8">
-        <v>0.45152657093515003</v>
+        <v>0.45187607368224109</v>
       </c>
     </row>
     <row r="9">
@@ -624,7 +624,7 @@
         <v>2018</v>
       </c>
       <c r="B9">
-        <v>0.45229760114705486</v>
+        <v>0.45230632619383604</v>
       </c>
     </row>
     <row r="10">
@@ -632,7 +632,7 @@
         <v>2019</v>
       </c>
       <c r="B10">
-        <v>0.46535045478865705</v>
+        <v>0.46535641588110904</v>
       </c>
     </row>
     <row r="11">
@@ -640,7 +640,7 @@
         <v>2020</v>
       </c>
       <c r="B11">
-        <v>0.46204877116646381</v>
+        <v>0.46203656399953613</v>
       </c>
     </row>
     <row r="12">
@@ -648,7 +648,7 @@
         <v>2021</v>
       </c>
       <c r="B12">
-        <v>0.46414907509722603</v>
+        <v>0.46415923362147143</v>
       </c>
     </row>
     <row r="13">
@@ -656,7 +656,7 @@
         <v>2022</v>
       </c>
       <c r="B13">
-        <v>0.46357452488896622</v>
+        <v>0.46358968623001989</v>
       </c>
     </row>
     <row r="14">
@@ -664,7 +664,7 @@
         <v>2023</v>
       </c>
       <c r="B14">
-        <v>0.4525317966921889</v>
+        <v>0.45193976910657391</v>
       </c>
     </row>
   </sheetData>
@@ -689,7 +689,7 @@
         <v>2011</v>
       </c>
       <c r="B2">
-        <v>0.42127446850781519</v>
+        <v>0.42127397982084658</v>
       </c>
     </row>
     <row r="3">
@@ -697,7 +697,7 @@
         <v>2012</v>
       </c>
       <c r="B3">
-        <v>0.41140297680864141</v>
+        <v>0.41139981807067022</v>
       </c>
     </row>
     <row r="4">
@@ -705,7 +705,7 @@
         <v>2013</v>
       </c>
       <c r="B4">
-        <v>0.42992468104303139</v>
+        <v>0.42997161789631533</v>
       </c>
     </row>
     <row r="5">
@@ -713,7 +713,7 @@
         <v>2014</v>
       </c>
       <c r="B5">
-        <v>0.43283704384710076</v>
+        <v>0.43275223152559544</v>
       </c>
     </row>
     <row r="6">
@@ -721,7 +721,7 @@
         <v>2015</v>
       </c>
       <c r="B6">
-        <v>0.44202836615462865</v>
+        <v>0.44202322948787881</v>
       </c>
     </row>
     <row r="7">
@@ -729,7 +729,7 @@
         <v>2016</v>
       </c>
       <c r="B7">
-        <v>0.44523637291596474</v>
+        <v>0.44517744844906476</v>
       </c>
     </row>
     <row r="8">
@@ -737,7 +737,7 @@
         <v>2017</v>
       </c>
       <c r="B8">
-        <v>0.45419556937786704</v>
+        <v>0.454197533517332</v>
       </c>
     </row>
     <row r="9">
@@ -745,7 +745,7 @@
         <v>2018</v>
       </c>
       <c r="B9">
-        <v>0.45065720087397249</v>
+        <v>0.45090560347589714</v>
       </c>
     </row>
     <row r="10">
@@ -753,7 +753,7 @@
         <v>2019</v>
       </c>
       <c r="B10">
-        <v>0.44371951862278519</v>
+        <v>0.44388496690103335</v>
       </c>
     </row>
     <row r="11">
@@ -761,7 +761,7 @@
         <v>2020</v>
       </c>
       <c r="B11">
-        <v>0.44281599996356591</v>
+        <v>0.44281420563924695</v>
       </c>
     </row>
     <row r="12">
@@ -769,7 +769,7 @@
         <v>2021</v>
       </c>
       <c r="B12">
-        <v>0.44498933731010126</v>
+        <v>0.44512593004149459</v>
       </c>
     </row>
     <row r="13">
@@ -777,7 +777,7 @@
         <v>2022</v>
       </c>
       <c r="B13">
-        <v>0.45292280255101874</v>
+        <v>0.45305412911862847</v>
       </c>
     </row>
     <row r="14">
@@ -785,7 +785,7 @@
         <v>2023</v>
       </c>
       <c r="B14">
-        <v>0.47013365426231118</v>
+        <v>0.47007709643136925</v>
       </c>
     </row>
   </sheetData>
@@ -810,7 +810,7 @@
         <v>2011</v>
       </c>
       <c r="B2">
-        <v>0.47583558016598038</v>
+        <v>0.47583369496353367</v>
       </c>
     </row>
     <row r="3">
@@ -818,7 +818,7 @@
         <v>2012</v>
       </c>
       <c r="B3">
-        <v>0.4614171678571814</v>
+        <v>0.46140025824213837</v>
       </c>
     </row>
     <row r="4">
@@ -826,7 +826,7 @@
         <v>2013</v>
       </c>
       <c r="B4">
-        <v>0.47274716778791298</v>
+        <v>0.47281039085967752</v>
       </c>
     </row>
     <row r="5">
@@ -834,7 +834,7 @@
         <v>2014</v>
       </c>
       <c r="B5">
-        <v>0.47961302057064198</v>
+        <v>0.47962800588710258</v>
       </c>
     </row>
     <row r="6">
@@ -842,7 +842,7 @@
         <v>2015</v>
       </c>
       <c r="B6">
-        <v>0.47737495825657933</v>
+        <v>0.47743094378514534</v>
       </c>
     </row>
     <row r="7">
@@ -850,7 +850,7 @@
         <v>2016</v>
       </c>
       <c r="B7">
-        <v>0.48187650507655377</v>
+        <v>0.48187432582112538</v>
       </c>
     </row>
     <row r="8">
@@ -858,7 +858,7 @@
         <v>2017</v>
       </c>
       <c r="B8">
-        <v>0.47220080042628554</v>
+        <v>0.47220076730665222</v>
       </c>
     </row>
     <row r="9">
@@ -866,7 +866,7 @@
         <v>2018</v>
       </c>
       <c r="B9">
-        <v>0.46183758332319952</v>
+        <v>0.46182800035797977</v>
       </c>
     </row>
     <row r="10">
@@ -874,7 +874,7 @@
         <v>2019</v>
       </c>
       <c r="B10">
-        <v>0.4705449351523025</v>
+        <v>0.47053750564137392</v>
       </c>
     </row>
     <row r="11">
@@ -882,7 +882,7 @@
         <v>2020</v>
       </c>
       <c r="B11">
-        <v>0.46481660419702481</v>
+        <v>0.46480459112038058</v>
       </c>
     </row>
     <row r="12">
@@ -890,7 +890,7 @@
         <v>2021</v>
       </c>
       <c r="B12">
-        <v>0.47764512230856598</v>
+        <v>0.47763860654562213</v>
       </c>
     </row>
     <row r="13">
@@ -898,7 +898,7 @@
         <v>2022</v>
       </c>
       <c r="B13">
-        <v>0.50993016077900999</v>
+        <v>0.50978801381886463</v>
       </c>
     </row>
     <row r="14">
@@ -906,7 +906,7 @@
         <v>2023</v>
       </c>
       <c r="B14">
-        <v>0.52898282992324175</v>
+        <v>0.52910064464416928</v>
       </c>
     </row>
   </sheetData>

</xml_diff>